<commit_message>
Update timeline with latest Excel data - 21 milestones
- Sync SGP_Milestones.xlsx with latest milestone descriptions
- Update HTML timeline with new Excel data
- 21 complete milestones from 2006-2026
- Ready for public access and display

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfQUztDgGAYhuwetw92SPH
</commit_message>
<xml_diff>
--- a/SGP_Milestones.xlsx
+++ b/SGP_Milestones.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -754,7 +754,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Felicitation of Sri Samavedam garu and Sri Goteti Srinivasa Rao garu; book launches including Srividhya GnanaDeepa Shikha</t>
+          <t>Felicitation of Sri Samavedam garu and Sri Goteti Srinivasa Rao garu; books launched Saparya kadambam, Anthardhara, Tyagaraja sourabham</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Concert by Sri Nihal garu</t>
+          <t>Concert by Sri Nihal garu &amp; team with rare kritis of Trinity of Music, Annamaya, Kshetrayya</t>
         </is>
       </c>
     </row>

</xml_diff>